<commit_message>
Add partner approval and onboarding workflow.
</commit_message>
<xml_diff>
--- a/D:\AutomationReports/AddPartner/2026-10-13.xlsx
+++ b/D:\AutomationReports/AddPartner/2026-10-13.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,281 +470,6 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>Execution Time</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TC003-1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>AddPartner</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Individual</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Individual: Locator.fill: Timeout 30000ms exceeded.
-Call log:
-  - waiting for get_by_test_id("dynamic-input-buisness_name").first
-  -     - locator resolved to &lt;input disabled type="text" name="buisness_name" data-testid="dynamic-input-buisness_name" placeholder="Enter business / entity name" class="h-11 admin-form-input rounded-lg border border-app-border px-3 text-sm text-app-foreground focus:outline-none focus:ring-2 focus:ring-app-input-focus/35 bg-gray-100 cursor-not-allowed text-gray-500"/&gt;
-  -     - fill("JOHN DOE INDUSTRIES")
-  -   - attempting fill action
-  -     2 × waiting for element to be visible, enabled and editable
-  -       - element is not enabled
-  -     - retrying fill action
-  -     - waiting 20ms
-  -     2 × waiting for element to be visible, enabled and editable
-  -       - element is not enabled
-  -     - retrying fill action
-  -       - waiting 100ms
-  -     46 × waiting for element to be visible, enabled and editable
-  -        - element is not enabled
-  -      - retrying fill action
-  -        - waiting 500ms
-  -     - waiting for element to be visible, enabled and editable
-  -   - element was detached from the DOM, retrying
-</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/email-availability/?email=nzrudo%40gmail.com | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/bank/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/gstin/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at&amp;email=nzrudo%40gmail.com | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/verify/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true =&gt; [{'id': '46690777-9e8f-41a2-8b98-3a125f0df31b', 'agent_type_name': 'Individual', 'field_code': 'account_holder_name', 'field_name': 'Account Holder Name', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': None, 'validation_message': None, 'placeholder': None, 'display_order': 60, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-17T16:20:18.624643+05:30', 'updated_at': '2026-09-29T23:24:46.403970+05:30', 'agent_type': 'ec8d7645-535d | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/email-availability/?email=nzrudo%40gmail.com =&gt; {'available': True} | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ =&gt; {'success': True, 'data': {'pan': 'ABCPV1234D', 'type': 'Individual', 'reference_id': 1429803, 'name_provided': '', 'registered_name': 'JOHN DOE', 'valid': True, 'message': 'PAN verified successfully', 'aadhaar_seeding_status': 'Y', 'last_updated_at': '01/01/2019', 'name_pan_card': 'JOHN DOE', 'pan_status': 'VALID', 'aadhaar_seeding_status_desc': 'Aadhaar is linked to PAN', 'pan_status_code': 'E', 'pan_status_desc': 'Existing and Valid'}} | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/bank/ =&gt; {'success': True, 'data': {'reference_id': 5240157, 'name_at_bank': 'JOHN DOE', 'bank_name': 'YES BANK', 'utr': None, 'city': 'MUMBAI', 'branch': 'SANTACRUZ, MUMBAI', 'micr': 400065001, 'name_match_score': None, 'name_match_result': None, 'account_status': 'VALID', 'account_status_code': 'ACCOUNT_IS_VALID', 'ifsc_details': {'bank': 'Yes Bank', 'ifsc': 'YESB0000262', 'micr': 400065001, 'nbin': None, 'address': 'GRND FLR, SAILESH BLDG, LINKING RD,, ERSTWHILE BENZER STORE AT LNKNG RD, NXT TO HDFC B | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/gstin/ =&gt; {'success': True, 'data': {'reference_id': 301571, 'GSTIN': '29AAICP2912R1ZR', 'legal_name_of_business': 'UJJIVAN SMALL FINANCE BANK LIMITED', 'trade_name_of_business': 'UJJIVAN SMALL FINANCE BANK', 'center_jurisdiction': 'I-A RANGE', 'state_jurisdiction': 'GUWAHATI - A - 1', 'date_of_registration': '2017-09-30', 'constitution_of_business': 'Public Limited Company', 'taxpayer_type': 'Regular', 'gst_in_status': 'Active', 'last_update_date': '2022-03-01', 'nature_of_business_activities': ['Retail  | POST 201 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/ =&gt; {'id': 'fe20b000-b862-4e7a-9202-5bf43f6b7354', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Individual', 'agent_channel_name': 'External Agent', 'referral_source_code': 'PR', 'referral_source_name': 'Existing Partner Referral', 'referral_source_is_code_required': True, 'verified_by_user': None, 'category': 'Partner', 'documents': [], 'agent_name': 'JOHN DOE', 'buisness_name': 'UJJIVAN SMALL FINANCE BANK LIMITED', 'agent_code': 'TPIBLRPR-00213', 'referral_code': ' | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true =&gt; [{'id': '3acedb4e-7fc5-4b8d-b083-2055850ca2a6', 'agent_type_name': 'Individual', 'document_code': 'aadhar_image', 'document_name': 'Aadhar Image', 'description': 'Aadhar Card', 'is_mandatory': True, 'is_corparate_mandatory': False, 'allowed_formats': 'pdf,jpg,jpeg,png', 'max_file_size_mb': 5, 'display_order': 2, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-26T16:36:11.016651+05:30', 'updated_at': '2026-09-26T16:36:11.016651+05:30', 'agent_type': 'ec8d7645-535d-4a02-a2e6-059609a6 | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/aadhar_image_30c468dd-873c-4d21-9d46-125ad6379dee.png', 'status': 'Draft', 'document': {'document_code': 'aadhar_image', 'document_name': 'Aadhar Image', 'name': 'Aadhar Image', 'field': 'aadhar_image', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/aadhar_image_30c468dd-873c-4d21-9d46-125ad6379dee.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/fe20b000-b862-4e7a-9202-5bf43f6b7354/aadhar_i | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/gst_image_corporate_0a2fafcc-3bc3-4f8a-b45d-4b7bba1b6dc9.png', 'status': 'Draft', 'document': {'document_code': 'gst_image_corporate', 'document_name': 'Corporate GST Certificate', 'name': 'Corporate GST Certificate', 'field': 'gst_image_corporate', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/gst_image_corporate_0a2fafcc-3bc3-4f8a-b45d-4b7bba1b6dc9.png', 'url': 'https://kyc-agents-documents.s3.amazo | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/pan_card_director_image_a589cb25-9110-48ec-8600-8103d30a1d11.png', 'status': 'Draft', 'document': {'document_code': 'pan_card_director_image', 'document_name': 'Director / Partner PAN Card', 'name': 'Director / Partner PAN Card', 'field': 'pan_card_director_image', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/pan_card_director_image_a589cb25-9110-48ec-8600-8103d30a1d11.png', 'url': 'https://kyc-agent | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/aadhar_card_director_image_adb15c4f-a2e3-4de5-b07e-bf0e70a8a173.png', 'status': 'Draft', 'document': {'document_code': 'aadhar_card_director_image', 'document_name': 'Director / Partner Aadhar Card', 'name': 'Director / Partner Aadhar Card', 'field': 'aadhar_card_director_image', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/aadhar_card_director_image_adb15c4f-a2e3-4de5-b07e-bf0e70a8a173.png', 'url':  | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/pan_image_4f06c934-2c51-4a23-9672-79e2f5b92a33.png', 'status': 'Draft', 'document': {'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/pan_image_4f06c934-2c51-4a23-9672-79e2f5b92a33.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/fe20b000-b862-4e7a-9202-5bf43f6b7354/pan_image_4f06c934-2c51-4a | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/uday_certificate_image_48117433-af71-4f6f-bcb7-ea29a1cef365.png', 'status': 'Draft', 'document': {'document_code': 'uday_certificate_image', 'document_name': 'Udyam / Uday Certificate', 'name': 'Udyam / Uday Certificate', 'field': 'uday_certificate_image', 's3_key': 'fe20b000-b862-4e7a-9202-5bf43f6b7354/uday_certificate_image_48117433-af71-4f6f-bcb7-ea29a1cef365.png', 'url': 'https://kyc-agents-document | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at =&gt; {'count': 256, 'page': 1, 'page_size': 20, 'total_pages': 13, 'next': 'http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_corporate=false&amp;is_verified=false&amp;ordering=-updated_at&amp;page=2&amp;page_size=20', 'previous': None, 'results': [{'id': 'fe20b000-b862-4e7a-9202-5bf43f6b7354', 'agent_code': 'TPIBLRPR-00213', 'agent_name': 'JOHN DOE', 'branch': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'branch_name': 'Adyar, Chennai', 'agent_type' | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at&amp;email=nzrudo%40gmail.com =&gt; {'count': 1, 'page': 1, 'page_size': 20, 'total_pages': 1, 'next': None, 'previous': None, 'results': [{'id': 'fe20b000-b862-4e7a-9202-5bf43f6b7354', 'agent_code': 'TPIBLRPR-00213', 'agent_name': 'JOHN DOE', 'branch': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'branch_name': 'Adyar, Chennai', 'agent_type': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'agent_type_name': 'Individual', 'category': 'Partner', 'email': 'nzrudo@gmail.com', 'created_at': '2026-10-13T18:35:21.181381+05:30', 'markup': False, 'st | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/ =&gt; {'id': 'fe20b000-b862-4e7a-9202-5bf43f6b7354', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Individual', 'agent_channel_name': 'External Agent', 'referral_source_code': 'PR', 'referral_source_name': 'Existing Partner Referral', 'referral_source_is_code_required': True, 'verified_by_user': None, 'category': 'Partner', 'documents': [{'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': 'fe20b000-b862-4e7a- | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true =&gt; [{'id': '46690777-9e8f-41a2-8b98-3a125f0df31b', 'agent_type_name': 'Individual', 'field_code': 'account_holder_name', 'field_name': 'Account Holder Name', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': None, 'validation_message': None, 'placeholder': None, 'display_order': 60, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-17T16:20:18.624643+05:30', 'updated_at': '2026-09-29T23:24:46.403970+05:30', 'agent_type': 'ec8d7645-535d | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true =&gt; [{'id': '3acedb4e-7fc5-4b8d-b083-2055850ca2a6', 'agent_type_name': 'Individual', 'document_code': 'aadhar_image', 'document_name': 'Aadhar Image', 'description': 'Aadhar Card', 'is_mandatory': True, 'is_corparate_mandatory': False, 'allowed_formats': 'pdf,jpg,jpeg,png', 'max_file_size_mb': 5, 'display_order': 2, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-26T16:36:11.016651+05:30', 'updated_at': '2026-09-26T16:36:11.016651+05:30', 'agent_type': 'ec8d7645-535d-4a02-a2e6-059609a6 | POST 400 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/verify/ =&gt; {'registered_mobile_number': 'Registered Mobile (Bank) is required before approval.', 'is_pan_verified': 'PAN must be verified before approval.'} | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/fe20b000-b862-4e7a-9202-5bf43f6b7354/ =&gt; {'id': 'fe20b000-b862-4e7a-9202-5bf43f6b7354', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Individual', 'agent_channel_name': 'External Agent', 'referral_source_code': 'PR', 'referral_source_name': 'Existing Partner Referral', 'referral_source_is_code_required': True, 'verified_by_user': None, 'category': 'Partner', 'documents': [{'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': 'fe20b000-b862-4e7a- | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true =&gt; [{'id': '46690777-9e8f-41a2-8b98-3a125f0df31b', 'agent_type_name': 'Individual', 'field_code': 'account_holder_name', 'field_name': 'Account Holder Name', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': None, 'validation_message': None, 'placeholder': None, 'display_order': 60, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-17T16:20:18.624643+05:30', 'updated_at': '2026-09-29T23:24:46.403970+05:30', 'agent_type': 'ec8d7645-535d | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=ec8d7645-535d-4a02-a2e6-059609a6cfe3&amp;is_active=true =&gt; [{'id': '46690777-9e8f-41a2-8b98-3a125f0df31b', 'agent_type_name': 'Individual', 'field_code': 'account_holder_name', 'field_name': 'Account Holder Name', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': None, 'validation_message': None, 'placeholder': None, 'display_order': 60, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-17T16:20:18.624643+05:30', 'updated_at': '2026-09-29T23:24:46.403970+05:30', 'agent_type': 'ec8d7645-535d | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ =&gt; {'success': True, 'data': {'pan': 'ABCPV1234D', 'type': 'Individual', 'reference_id': 1429804, 'name_provided': '', 'registered_name': 'JOHN DOE', 'valid': True, 'message': 'PAN verified successfully', 'aadhaar_seeding_status': 'Y', 'last_updated_at': '01/01/2019', 'name_pan_card': 'JOHN DOE', 'pan_status': 'VALID', 'aadhaar_seeding_status_desc': 'Aadhaar is linked to PAN', 'pan_status_code': 'E', 'pan_status_desc': 'Existing and Valid'}} | PATCH 200 http://p</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>64.13</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>reports/screenshots/test_add_partner.png</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2026-10-13 18:36:05</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TC003-2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>AddPartner</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>LLP</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LLP: Locator.fill: Timeout 30000ms exceeded.
-Call log:
-  - waiting for get_by_test_id("dynamic-input-buisness_name").first
-  -     - locator resolved to &lt;input disabled type="text" name="buisness_name" data-testid="dynamic-input-buisness_name" placeholder="Enter business / entity name" class="h-11 admin-form-input rounded-lg border border-app-border px-3 text-sm text-app-foreground focus:outline-none focus:ring-2 focus:ring-app-input-focus/35 bg-gray-100 cursor-not-allowed text-gray-500"/&gt;
-  -     - fill("JOHN DOE LLP")
-  -   - attempting fill action
-  -     2 × waiting for element to be visible, enabled and editable
-  -       - element is not enabled
-  -     - retrying fill action
-  -     - waiting 20ms
-  -     2 × waiting for element to be visible, enabled and editable
-  -       - element is not enabled
-  -     - retrying fill action
-  -       - waiting 100ms
-  -     60 × waiting for element to be visible, enabled and editable
-  -        - element is not enabled
-  -      - retrying fill action
-  -        - waiting 500ms
-</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/email-availability/?email=rf7naf%40gmail.com | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/bank/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/gstin/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at&amp;email=rf7naf%40gmail.com | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/verify/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true =&gt; [{'id': '28f6810c-b7a3-4bf6-b3f9-0b8c8ae324b1', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'field_code': 'bank_account_number', 'field_name': 'Bank Account Number', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': '^[0-9]{9,18}$', 'validation_message': 'Enter a valid bank account number.', 'placeholder': None, 'display_order': 40, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:50.867476+05:30', 'updated_a | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/email-availability/?email=rf7naf%40gmail.com =&gt; {'available': True} | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ =&gt; {'success': True, 'data': {'pan': 'ABCPV1234D', 'type': 'Individual', 'reference_id': 1429805, 'name_provided': '', 'registered_name': 'JOHN DOE', 'valid': True, 'message': 'PAN verified successfully', 'aadhaar_seeding_status': 'Y', 'last_updated_at': '01/01/2019', 'name_pan_card': 'JOHN DOE', 'pan_status': 'VALID', 'aadhaar_seeding_status_desc': 'Aadhaar is linked to PAN', 'pan_status_code': 'E', 'pan_status_desc': 'Existing and Valid'}} | POST 502 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/bank/ =&gt; {'success': False, 'error': '422 Client Error: Unprocessable Entity for url: https://sandbox.cashfree.com/verification/bank-account/sync', 'type': 'API_ERROR', 'details': {'type': 'validation_error', 'code': 'failed_at_bank', 'message': 'failed at bank.', 'error': {'reference_id': '5240160'}}} | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/gstin/ =&gt; {'success': True, 'data': {'reference_id': 301572, 'GSTIN': '29AAICP2912R1ZR', 'legal_name_of_business': 'UJJIVAN SMALL FINANCE BANK LIMITED', 'trade_name_of_business': 'UJJIVAN SMALL FINANCE BANK', 'center_jurisdiction': 'I-A RANGE', 'state_jurisdiction': 'GUWAHATI - A - 1', 'date_of_registration': '2017-09-30', 'constitution_of_business': 'Public Limited Company', 'taxpayer_type': 'Regular', 'gst_in_status': 'Active', 'last_update_date': '2022-03-01', 'nature_of_business_activities': ['Retail  | POST 201 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/ =&gt; {'id': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'agent_channel_name': 'Internal Agent', 'referral_source_code': 'CR', 'referral_source_name': 'Corporate Referral', 'referral_source_is_code_required': False, 'verified_by_user': None, 'category': 'Partner', 'documents': [], 'agent_name': 'JOHN DOE', 'buisness_name': 'UJJIVAN SMALL FINANCE BANK LIMITED', 'agent_code': 'LLPBLRCR-00214', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true =&gt; [{'id': '13122e0f-9bf7-4184-8eac-8e3cb09ed2a3', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'document_code': 'pan_image', 'document_name': 'PAN Image', 'description': 'PAN Card', 'is_mandatory': True, 'is_corparate_mandatory': False, 'allowed_formats': 'pdf,jpg,jpeg,png', 'max_file_size_mb': 5, 'display_order': 1, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-26T16:36:11.016651+05:30', 'updated_at': '2026-09-26T16:36:11.016651+05:30', 'agent_type': '0defce87-62f8-46 | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/pan_image_9990aadb-c4be-439b-9733-f2126acb8cba.png', 'status': 'Draft', 'document': {'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/pan_image_9990aadb-c4be-439b-9733-f2126acb8cba.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/pan_image_9990aadb-c4be-43 | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/aadhar_image_e31230ab-b6e2-4498-bf7a-2608bd8d6419.png', 'status': 'Draft', 'document': {'document_code': 'aadhar_image', 'document_name': 'Aadhar Image', 'name': 'Aadhar Image', 'field': 'aadhar_image', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/aadhar_image_e31230ab-b6e2-4498-bf7a-2608bd8d6419.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/aadhar_i | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/pan_card_director_image_6f247b94-acef-4e66-8354-f4368a29c8f0.png', 'status': 'Draft', 'document': {'document_code': 'pan_card_director_image', 'document_name': 'Director / Partner PAN Card', 'name': 'Director / Partner PAN Card', 'field': 'pan_card_director_image', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/pan_card_director_image_6f247b94-acef-4e66-8354-f4368a29c8f0.png', 'url': 'https://kyc-agent | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/llp_certificate_72bdb150-b9cf-49d1-8666-0cc9d6f4336f.png', 'status': 'Draft', 'document': {'document_code': 'llp_certificate', 'document_name': 'LLP Certificate', 'name': 'LLP Certificate', 'field': 'llp_certificate', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/llp_certificate_72bdb150-b9cf-49d1-8666-0cc9d6f4336f.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/f0e24b79-aea4-4b9e-b90c-8a7 | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/gst_image_corporate_84823a9d-9b19-4883-a2f4-a4fe9b75d081.png', 'status': 'Draft', 'document': {'document_code': 'gst_image_corporate', 'document_name': 'Corporate GST Certificate', 'name': 'Corporate GST Certificate', 'field': 'gst_image_corporate', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/gst_image_corporate_84823a9d-9b19-4883-a2f4-a4fe9b75d081.png', 'url': 'https://kyc-agents-documents.s3.amazo | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/llp_agreement_2d1722c9-e887-47d8-ab12-cdaae4575bfa.png', 'status': 'Draft', 'document': {'document_code': 'llp_agreement', 'document_name': 'LLP Agreement', 'name': 'LLP Agreement', 'field': 'llp_agreement', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/llp_agreement_2d1722c9-e887-47d8-ab12-cdaae4575bfa.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/ll | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/aadhar_card_director_image_77dd8665-7b22-4103-bcfa-938a25514d9a.png', 'status': 'Draft', 'document': {'document_code': 'aadhar_card_director_image', 'document_name': 'Director / Partner Aadhar Card', 'name': 'Director / Partner Aadhar Card', 'field': 'aadhar_card_director_image', 's3_key': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc/aadhar_card_director_image_77dd8665-7b22-4103-bcfa-938a25514d9a.png', 'url':  | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at =&gt; {'count': 257, 'page': 1, 'page_size': 20, 'total_pages': 13, 'next': 'http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_corporate=false&amp;is_verified=false&amp;ordering=-updated_at&amp;page=2&amp;page_size=20', 'previous': None, 'results': [{'id': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc', 'agent_code': 'LLPBLRCR-00214', 'agent_name': 'JOHN DOE', 'branch': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'branch_name': 'Adyar, Chennai', 'agent_type' | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at&amp;email=rf7naf%40gmail.com =&gt; {'count': 1, 'page': 1, 'page_size': 20, 'total_pages': 1, 'next': None, 'previous': None, 'results': [{'id': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc', 'agent_code': 'LLPBLRCR-00214', 'agent_name': 'JOHN DOE', 'branch': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'branch_name': 'Adyar, Chennai', 'agent_type': '0defce87-62f8-46f4-913e-fe0b9dfd5017', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'category': 'Partner', 'email': 'rf7naf@gmail.com', 'created_at': '2026-10-13T18:36:24.553883+05: | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/ =&gt; {'id': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'agent_channel_name': 'Internal Agent', 'referral_source_code': 'CR', 'referral_source_name': 'Corporate Referral', 'referral_source_is_code_required': False, 'verified_by_user': None, 'category': 'Partner', 'documents': [{'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': ' | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true =&gt; [{'id': '28f6810c-b7a3-4bf6-b3f9-0b8c8ae324b1', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'field_code': 'bank_account_number', 'field_name': 'Bank Account Number', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': '^[0-9]{9,18}$', 'validation_message': 'Enter a valid bank account number.', 'placeholder': None, 'display_order': 40, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:50.867476+05:30', 'updated_a | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true =&gt; [{'id': '13122e0f-9bf7-4184-8eac-8e3cb09ed2a3', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'document_code': 'pan_image', 'document_name': 'PAN Image', 'description': 'PAN Card', 'is_mandatory': True, 'is_corparate_mandatory': False, 'allowed_formats': 'pdf,jpg,jpeg,png', 'max_file_size_mb': 5, 'display_order': 1, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-26T16:36:11.016651+05:30', 'updated_at': '2026-09-26T16:36:11.016651+05:30', 'agent_type': '0defce87-62f8-46 | POST 400 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/verify/ =&gt; {'registered_mobile_number': 'Registered Mobile (Bank) is required before approval.', 'is_pan_verified': 'PAN must be verified before approval.', 'is_bank_details_verified': 'Bank details must be verified before approval.'} | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/f0e24b79-aea4-4b9e-b90c-8a73604a93bc/ =&gt; {'id': 'f0e24b79-aea4-4b9e-b90c-8a73604a93bc', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'agent_channel_name': 'Internal Agent', 'referral_source_code': 'CR', 'referral_source_name': 'Corporate Referral', 'referral_source_is_code_required': False, 'verified_by_user': None, 'category': 'Partner', 'documents': [{'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': ' | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true =&gt; [{'id': '28f6810c-b7a3-4bf6-b3f9-0b8c8ae324b1', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'field_code': 'bank_account_number', 'field_name': 'Bank Account Number', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': '^[0-9]{9,18}$', 'validation_message': 'Enter a valid bank account number.', 'placeholder': None, 'display_order': 40, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:50.867476+05:30', 'updated_a | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=0defce87-62f8-46f4-913e-fe0b9dfd5017&amp;is_active=true =&gt; [{'id': '28f6810c-b7a3-4bf6-b3f9-0b8c8ae324b1', 'agent_type_name': 'Limited Liability Partnership (LLP)', 'field_code': 'bank_account_number', 'field_name': 'Bank Account Number', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': '^[0-9]{9,18}$', 'validation_message': 'Enter a valid bank account number.', 'placeholder': None, 'display_order': 40, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:50.867476+05:30', 'updated_a | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>64.03</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>reports/screenshots/test_add_partner.png</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2026-10-13 18:37:09</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>TC003-3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>AddPartner</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Partnership Firm</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partnership Firm: Locator.fill: Timeout 30000ms exceeded.
-Call log:
-  - waiting for get_by_test_id("dynamic-input-buisness_name").first
-  -     - locator resolved to &lt;input disabled type="text" name="buisness_name" data-testid="dynamic-input-buisness_name" placeholder="Enter business / entity name" class="h-11 admin-form-input rounded-lg border border-app-border px-3 text-sm text-app-foreground focus:outline-none focus:ring-2 focus:ring-app-input-focus/35 bg-gray-100 cursor-not-allowed text-gray-500"/&gt;
-  -     - fill("JOHN DOE PARTNERSHIP")
-  -   - attempting fill action
-  -     2 × waiting for element to be visible, enabled and editable
-  -       - element is not enabled
-  -     - retrying fill action
-  -     - waiting 20ms
-  -     2 × waiting for element to be visible, enabled and editable
-  -       - element is not enabled
-  -     - retrying fill action
-  -       - waiting 100ms
-  -     60 × waiting for element to be visible, enabled and editable
-  -        - element is not enabled
-  -      - retrying fill action
-  -        - waiting 500ms
-</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/email-availability/?email=ll6sxk%40gmail.com | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/bank/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/gstin/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at&amp;email=ll6sxk%40gmail.com | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/verify/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true =&gt; [{'id': '21033248-6d32-4592-85c9-62c38c61a278', 'agent_type_name': 'Partnership Firm', 'field_code': 'gst_number', 'field_name': 'GSTIN Number', 'section': 'profile', 'input_type': 'text', 'is_required': False, 'validation_regex': '^[0-9]{2}[A-Z]{5}[0-9]{4}[A-Z][1-9A-Z]Z[0-9A-Z]$', 'validation_message': 'Enter a valid GSTIN number.', 'placeholder': None, 'display_order': 30, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:49.096791+05:30', 'updated_at': '2 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/email-availability/?email=ll6sxk%40gmail.com =&gt; {'available': True} | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ =&gt; {'success': True, 'data': {'pan': 'ABCPV1234D', 'type': 'Individual', 'reference_id': 1429807, 'name_provided': '', 'registered_name': 'JOHN DOE', 'valid': True, 'message': 'PAN verified successfully', 'aadhaar_seeding_status': 'Y', 'last_updated_at': '01/01/2019', 'name_pan_card': 'JOHN DOE', 'pan_status': 'VALID', 'aadhaar_seeding_status_desc': 'Aadhaar is linked to PAN', 'pan_status_code': 'E', 'pan_status_desc': 'Existing and Valid'}} | POST 502 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/bank/ =&gt; {'success': False, 'error': '422 Client Error: Unprocessable Entity for url: https://sandbox.cashfree.com/verification/bank-account/sync', 'type': 'API_ERROR', 'details': {'type': 'validation_error', 'code': 'failed_at_bank', 'message': 'failed at bank.', 'error': {'reference_id': '5240162'}}} | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/gstin/ =&gt; {'success': True, 'data': {'reference_id': 301573, 'GSTIN': '29AAICP2912R1ZR', 'legal_name_of_business': 'UJJIVAN SMALL FINANCE BANK LIMITED', 'trade_name_of_business': 'UJJIVAN SMALL FINANCE BANK', 'center_jurisdiction': 'I-A RANGE', 'state_jurisdiction': 'GUWAHATI - A - 1', 'date_of_registration': '2017-09-30', 'constitution_of_business': 'Public Limited Company', 'taxpayer_type': 'Regular', 'gst_in_status': 'Active', 'last_update_date': '2022-03-01', 'nature_of_business_activities': ['Retail  | POST 201 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/ =&gt; {'id': 'df90690a-9af6-4b7e-b281-d3807200a91b', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Partnership Firm', 'agent_channel_name': 'External Agent', 'referral_source_code': 'DI', 'referral_source_name': 'Direct/Walk-in', 'referral_source_is_code_required': False, 'verified_by_user': None, 'category': 'Partner', 'documents': [], 'agent_name': 'JOHN DOE', 'buisness_name': 'UJJIVAN SMALL FINANCE BANK LIMITED', 'agent_code': 'TPFBLRDI-00215', 'referral_code': None, | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true =&gt; [{'id': '182cb887-ec1c-4f68-a81e-f2918674b9be', 'agent_type_name': 'Partnership Firm', 'document_code': 'pan_image', 'document_name': 'PAN Image', 'description': 'PAN Card', 'is_mandatory': True, 'is_corparate_mandatory': False, 'allowed_formats': 'pdf,jpg,jpeg,png', 'max_file_size_mb': 5, 'display_order': 1, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-26T16:36:11.016651+05:30', 'updated_at': '2026-09-26T16:36:11.016651+05:30', 'agent_type': '7362c6a4-5b75-42d4-9cf6-a8ccedf512c | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/pan_image_b164fc67-f7c5-48f0-b32a-4dc9862d20d9.png', 'status': 'Draft', 'document': {'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/pan_image_b164fc67-f7c5-48f0-b32a-4dc9862d20d9.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/df90690a-9af6-4b7e-b281-d3807200a91b/pan_image_b164fc67-f7c5-48 | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/llp_agreement_3b169f00-6b01-42f6-99fe-78f0fc6eb474.png', 'status': 'Draft', 'document': {'document_code': 'llp_agreement', 'document_name': 'LLP Agreement', 'name': 'LLP Agreement', 'field': 'llp_agreement', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/llp_agreement_3b169f00-6b01-42f6-99fe-78f0fc6eb474.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/df90690a-9af6-4b7e-b281-d3807200a91b/ll | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/aadhar_image_1fb880db-add6-4ca2-8626-fbeba3ea0ed5.png', 'status': 'Draft', 'document': {'document_code': 'aadhar_image', 'document_name': 'Aadhar Image', 'name': 'Aadhar Image', 'field': 'aadhar_image', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/aadhar_image_1fb880db-add6-4ca2-8626-fbeba3ea0ed5.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/df90690a-9af6-4b7e-b281-d3807200a91b/aadhar_i | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/pan_card_director_image_d99d958e-b77e-4a77-a101-d4529517d934.png', 'status': 'Draft', 'document': {'document_code': 'pan_card_director_image', 'document_name': 'Director / Partner PAN Card', 'name': 'Director / Partner PAN Card', 'field': 'pan_card_director_image', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/pan_card_director_image_d99d958e-b77e-4a77-a101-d4529517d934.png', 'url': 'https://kyc-agent | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/aadhar_card_director_image_193ced70-a547-428c-bd8e-4fb46010cdbb.png', 'status': 'Draft', 'document': {'document_code': 'aadhar_card_director_image', 'document_name': 'Director / Partner Aadhar Card', 'name': 'Director / Partner Aadhar Card', 'field': 'aadhar_card_director_image', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/aadhar_card_director_image_193ced70-a547-428c-bd8e-4fb46010cdbb.png', 'url':  | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/partnership_deed_c10251f5-6e15-428b-83a9-19843e8655ca.png', 'status': 'Draft', 'document': {'document_code': 'partnership_deed', 'document_name': 'Partnership Deed', 'name': 'Partnership Deed', 'field': 'partnership_deed', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/partnership_deed_c10251f5-6e15-428b-83a9-19843e8655ca.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/df90690a-9af6-4b7e-b2 | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/gst_image_corporate_b8b370c2-138c-473e-a62e-90b46e5c3f6b.png', 'status': 'Draft', 'document': {'document_code': 'gst_image_corporate', 'document_name': 'Corporate GST Certificate', 'name': 'Corporate GST Certificate', 'field': 'gst_image_corporate', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/gst_image_corporate_b8b370c2-138c-473e-a62e-90b46e5c3f6b.png', 'url': 'https://kyc-agents-documents.s3.amazo | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/llp_certificate_1b899d45-24b9-48e0-be3e-f00a8fe2f678.png', 'status': 'Draft', 'document': {'document_code': 'llp_certificate', 'document_name': 'LLP Certificate', 'name': 'LLP Certificate', 'field': 'llp_certificate', 's3_key': 'df90690a-9af6-4b7e-b281-d3807200a91b/llp_certificate_1b899d45-24b9-48e0-be3e-f00a8fe2f678.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/df90690a-9af6-4b7e-b281-d38 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at =&gt; {'count': 258, 'page': 1, 'page_size': 20, 'total_pages': 13, 'next': 'http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_corporate=false&amp;is_verified=false&amp;ordering=-updated_at&amp;page=2&amp;page_size=20', 'previous': None, 'results': [{'id': 'df90690a-9af6-4b7e-b281-d3807200a91b', 'agent_code': 'TPFBLRDI-00215', 'agent_name': 'JOHN DOE', 'branch': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'branch_name': 'Adyar, Chennai', 'agent_type' | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; Could not parse response | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at =&gt; {'count': 258, 'page': 1, 'page_size': 20, 'total_pages': 13, 'next': 'http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_corporate=false&amp;is_verified=false&amp;ordering=-updated_at&amp;page=2&amp;page_size=20', 'previous': None, 'results': [{'id': 'df90690a-9af6-4b7e-b281-d3807200a91b', 'agent_code': 'TPFBLRDI-00215', 'agent_name': 'JOHN DOE', 'branch': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'branch_name': 'Adyar, Chennai', 'agent_type' | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at&amp;email=ll6sxk%40gmail.com =&gt; {'count': 1, 'page': 1, 'page_size': 20, 'total_pages': 1, 'next': None, 'previous': None, 'results': [{'id': 'df90690a-9af6-4b7e-b281-d3807200a91b', 'agent_code': 'TPFBLRDI-00215', 'agent_name': 'JOHN DOE', 'branch': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'branch_name': 'Adyar, Chennai', 'agent_type': '7362c6a4-5b75-42d4-9cf6-a8ccedf512cb', 'agent_type_name': 'Partnership Firm', 'category': 'Partner', 'email': 'll6sxk@gmail.com', 'created_at': '2026-10-13T18:37:29.202590+05:30', 'markup': Fals | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/ =&gt; {'id': 'df90690a-9af6-4b7e-b281-d3807200a91b', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Partnership Firm', 'agent_channel_name': 'External Agent', 'referral_source_code': 'DI', 'referral_source_name': 'Direct/Walk-in', 'referral_source_is_code_required': False, 'verified_by_user': None, 'category': 'Partner', 'documents': [{'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': 'df90690a-9af6-4b7e-b281 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true =&gt; [{'id': '21033248-6d32-4592-85c9-62c38c61a278', 'agent_type_name': 'Partnership Firm', 'field_code': 'gst_number', 'field_name': 'GSTIN Number', 'section': 'profile', 'input_type': 'text', 'is_required': False, 'validation_regex': '^[0-9]{2}[A-Z]{5}[0-9]{4}[A-Z][1-9A-Z]Z[0-9A-Z]$', 'validation_message': 'Enter a valid GSTIN number.', 'placeholder': None, 'display_order': 30, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:49.096791+05:30', 'updated_at': '2 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true =&gt; [{'id': '182cb887-ec1c-4f68-a81e-f2918674b9be', 'agent_type_name': 'Partnership Firm', 'document_code': 'pan_image', 'document_name': 'PAN Image', 'description': 'PAN Card', 'is_mandatory': True, 'is_corparate_mandatory': False, 'allowed_formats': 'pdf,jpg,jpeg,png', 'max_file_size_mb': 5, 'display_order': 1, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-26T16:36:11.016651+05:30', 'updated_at': '2026-09-26T16:36:11.016651+05:30', 'agent_type': '7362c6a4-5b75-42d4-9cf6-a8ccedf512c | POST 400 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/verify/ =&gt; {'registered_mobile_number': 'Registered Mobile (Bank) is required before approval.', 'is_pan_verified': 'PAN must be verified before approval.', 'is_bank_details_verified': 'Bank details must be verified before approval.'} | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/df90690a-9af6-4b7e-b281-d3807200a91b/ =&gt; {'id': 'df90690a-9af6-4b7e-b281-d3807200a91b', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Partnership Firm', 'agent_channel_name': 'External Agent', 'referral_source_code': 'DI', 'referral_source_name': 'Direct/Walk-in', 'referral_source_is_code_required': False, 'verified_by_user': None, 'category': 'Partner', 'documents': [{'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': 'df90690a-9af6-4b7e-b281 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=7362c6a4-5b75-42d4-9cf6-a8ccedf512cb&amp;is_active=true =&gt; [{'id': '21033248-6d32-4592-85c9-62c38c61a278', 'agent_type_name': 'Partnership Firm', 'field_code': 'gst_number', 'field_name': 'GSTIN Number', 'section': 'profile', 'input_type': 'text', 'is_required': False, 'validation_regex': '^[0-9]{2}[A-Z]{5}[0-9]{4}[A-Z][1-9A-Z]Z[0-9A-Z]$', 'validation_message': 'Enter a valid GSTIN number.', 'placeholder': None, 'display_order': 30, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:49.096791+05:30', 'updated_at': '2 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa4</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>67.54000000000001</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>reports/screenshots/test_add_partner.png</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>2026-10-13 18:38:17</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>TC003-4</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>AddPartner</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Private Limited Company</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Private Limited Company: Locator.fill: Timeout 30000ms exceeded.
-Call log:
-  - waiting for get_by_test_id("dynamic-input-buisness_name").first
-  -     - locator resolved to &lt;input disabled type="text" name="buisness_name" data-testid="dynamic-input-buisness_name" placeholder="Enter business / entity name" class="h-11 admin-form-input rounded-lg border border-app-border px-3 text-sm text-app-foreground focus:outline-none focus:ring-2 focus:ring-app-input-focus/35 bg-gray-100 cursor-not-allowed text-gray-500"/&gt;
-  -     - fill("JOHN DOE PRIVATE LIMITED")
-  -   - attempting fill action
-  -     2 × waiting for element to be visible, enabled and editable
-  -       - element is not enabled
-  -     - retrying fill action
-  -     - waiting 20ms
-  -     2 × waiting for element to be visible, enabled and editable
-  -       - element is not enabled
-  -     - retrying fill action
-  -       - waiting 100ms
-  -     60 × waiting for element to be visible, enabled and editable
-  -        - element is not enabled
-  -      - retrying fill action
-  -        - waiting 500ms
-</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/email-availability/?email=atbo0c%40gmail.com | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/bank/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/gstin/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at&amp;email=atbo0c%40gmail.com | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/verify/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ | http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true =&gt; [{'id': '10bea8fd-2c9c-4703-9789-486491aa2e49', 'agent_type_name': 'Private Limited Company', 'field_code': 'cin_llpin', 'field_name': 'CIN / LLPIN Number', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': None, 'validation_message': None, 'placeholder': None, 'display_order': 90, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:53.590171+05:30', 'updated_at': '2026-09-29T23:24:53.590190+05:30', 'agent_type': '22e700fe-df | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/email-availability/?email=atbo0c%40gmail.com =&gt; {'available': True} | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/pan-full/ =&gt; {'success': True, 'data': {'pan': 'ABCPV1234D', 'type': 'Individual', 'reference_id': 1429811, 'name_provided': '', 'registered_name': 'JOHN DOE', 'valid': True, 'message': 'PAN verified successfully', 'aadhaar_seeding_status': 'Y', 'last_updated_at': '01/01/2019', 'name_pan_card': 'JOHN DOE', 'pan_status': 'VALID', 'aadhaar_seeding_status_desc': 'Aadhaar is linked to PAN', 'pan_status_code': 'E', 'pan_status_desc': 'Existing and Valid'}} | POST 502 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/bank/ =&gt; {'success': False, 'error': '422 Client Error: Unprocessable Entity for url: https://sandbox.cashfree.com/verification/bank-account/sync', 'type': 'API_ERROR', 'details': {'type': 'validation_error', 'code': 'failed_at_bank', 'message': 'failed at bank.', 'error': {'reference_id': '5240163'}}} | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/cashfree-verification/verify/gstin/ =&gt; {'success': True, 'data': {'reference_id': 301574, 'GSTIN': '29AAICP2912R1ZR', 'legal_name_of_business': 'UJJIVAN SMALL FINANCE BANK LIMITED', 'trade_name_of_business': 'UJJIVAN SMALL FINANCE BANK', 'center_jurisdiction': 'I-A RANGE', 'state_jurisdiction': 'GUWAHATI - A - 1', 'date_of_registration': '2017-09-30', 'constitution_of_business': 'Public Limited Company', 'taxpayer_type': 'Regular', 'gst_in_status': 'Active', 'last_update_date': '2022-03-01', 'nature_of_business_activities': ['Retail  | POST 201 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/ =&gt; {'id': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Private Limited Company', 'agent_channel_name': 'Internal Agent', 'referral_source_code': 'IN', 'referral_source_name': 'Internal (Sales Team)', 'referral_source_is_code_required': False, 'verified_by_user': None, 'category': 'Partner', 'documents': [], 'agent_name': 'JOHN DOE', 'buisness_name': 'UJJIVAN SMALL FINANCE BANK LIMITED', 'agent_code': 'PLCBLRIN-00216', 'referra | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true =&gt; [{'id': '07a9ba65-19f9-4f04-9277-536b6feadd97', 'agent_type_name': 'Private Limited Company', 'document_code': 'aadhar_card_director_image', 'document_name': 'Director / Partner Aadhar Card', 'description': 'Director / Partner Aadhar Card', 'is_mandatory': True, 'is_corparate_mandatory': False, 'allowed_formats': 'pdf,jpg,jpeg,png', 'max_file_size_mb': 5, 'display_order': 4, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-26T16:36:11.016651+05:30', 'updated_at': '2026-09-26T16:36:1 | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/aadhar_card_director_image_99230aad-c2aa-4e4c-b936-e13a058cf0ea.png', 'status': 'Draft', 'document': {'document_code': 'aadhar_card_director_image', 'document_name': 'Director / Partner Aadhar Card', 'name': 'Director / Partner Aadhar Card', 'field': 'aadhar_card_director_image', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/aadhar_card_director_image_99230aad-c2aa-4e4c-b936-e13a058cf0ea.png', 'url':  | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/aadhar_image_38191700-4b20-4419-9b75-f3896d95dc96.png', 'status': 'Draft', 'document': {'document_code': 'aadhar_image', 'document_name': 'Aadhar Image', 'name': 'Aadhar Image', 'field': 'aadhar_image', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/aadhar_image_38191700-4b20-4419-9b75-f3896d95dc96.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/aadhar_i | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/gst_image_corporate_ae68b9de-0697-4527-92ef-9dc12c62f8c1.png', 'status': 'Draft', 'document': {'document_code': 'gst_image_corporate', 'document_name': 'Corporate GST Certificate', 'name': 'Corporate GST Certificate', 'field': 'gst_image_corporate', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/gst_image_corporate_ae68b9de-0697-4527-92ef-9dc12c62f8c1.png', 'url': 'https://kyc-agents-documents.s3.amazo | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/moa_image_3a30a504-02b0-4409-82e7-afd9581795b8.png', 'status': 'Draft', 'document': {'document_code': 'moa_image', 'document_name': 'MOA', 'name': 'MOA', 'field': 'moa_image', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/moa_image_3a30a504-02b0-4409-82e7-afd9581795b8.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/moa_image_3a30a504-02b0-4409-82e7-afd9 | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/certificate_of_incorporation_c62b857c-4fc6-4595-b1f1-14992985e037.png', 'status': 'Draft', 'document': {'document_code': 'certificate_of_incorporation', 'document_name': 'Certificate of Incorporation', 'name': 'Certificate of Incorporation', 'field': 'certificate_of_incorporation', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/certificate_of_incorporation_c62b857c-4fc6-4595-b1f1-14992985e037.png', 'ur | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/aoa_image_f79af581-0ef9-4d03-bf11-349e48b37be3.png', 'status': 'Draft', 'document': {'document_code': 'aoa_image', 'document_name': 'AOA', 'name': 'AOA', 'field': 'aoa_image', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/aoa_image_f79af581-0ef9-4d03-bf11-349e48b37be3.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/aoa_image_f79af581-0ef9-4d03-bf11-349e | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/pan_card_director_image_5c891c7d-b620-4650-8201-c11d6503ae4e.png', 'status': 'Draft', 'document': {'document_code': 'pan_card_director_image', 'document_name': 'Director / Partner PAN Card', 'name': 'Director / Partner PAN Card', 'field': 'pan_card_director_image', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/pan_card_director_image_5c891c7d-b620-4650-8201-c11d6503ae4e.png', 'url': 'https://kyc-agent | POST 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/upload-document/ =&gt; {'message': 'Document uploaded successfully', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/pan_image_4b7055b6-2542-4e03-9056-16ec9503d867.png', 'status': 'Draft', 'document': {'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/pan_image_4b7055b6-2542-4e03-9056-16ec9503d867.png', 'url': 'https://kyc-agents-documents.s3.amazonaws.com/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/pan_image_4b7055b6-2542-4e | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/ =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at =&gt; {'count': 259, 'page': 1, 'page_size': 20, 'total_pages': 13, 'next': 'http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_corporate=false&amp;is_verified=false&amp;ordering=-updated_at&amp;page=2&amp;page_size=20', 'previous': None, 'results': [{'id': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a', 'agent_code': 'PLCBLRIN-00216', 'agent_name': 'JOHN DOE', 'branch': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'branch_name': 'Adyar, Chennai', 'agent_type' | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/partners-v1/?is_verified=false&amp;is_corporate=false&amp;page=1&amp;page_size=20&amp;ordering=-updated_at&amp;email=atbo0c%40gmail.com =&gt; {'count': 1, 'page': 1, 'page_size': 20, 'total_pages': 1, 'next': None, 'previous': None, 'results': [{'id': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a', 'agent_code': 'PLCBLRIN-00216', 'agent_name': 'JOHN DOE', 'branch': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'branch_name': 'Adyar, Chennai', 'agent_type': '22e700fe-df45-41b6-b72a-10a3506437f7', 'agent_type_name': 'Private Limited Company', 'category': 'Partner', 'email': 'atbo0c@gmail.com', 'created_at': '2026-10-13T18:38:36.205162+05:30', 'markup | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/ =&gt; {'id': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Private Limited Company', 'agent_channel_name': 'Internal Agent', 'referral_source_code': 'IN', 'referral_source_name': 'Internal (Sales Team)', 'referral_source_is_code_required': False, 'verified_by_user': None, 'category': 'Partner', 'documents': [{'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': '17bcd4d6- | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-documents/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true =&gt; [{'id': '07a9ba65-19f9-4f04-9277-536b6feadd97', 'agent_type_name': 'Private Limited Company', 'document_code': 'aadhar_card_director_image', 'document_name': 'Director / Partner Aadhar Card', 'description': 'Director / Partner Aadhar Card', 'is_mandatory': True, 'is_corparate_mandatory': False, 'allowed_formats': 'pdf,jpg,jpeg,png', 'max_file_size_mb': 5, 'display_order': 4, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-26T16:36:11.016651+05:30', 'updated_at': '2026-09-26T16:36:1 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true =&gt; [{'id': '10bea8fd-2c9c-4703-9789-486491aa2e49', 'agent_type_name': 'Private Limited Company', 'field_code': 'cin_llpin', 'field_name': 'CIN / LLPIN Number', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': None, 'validation_message': None, 'placeholder': None, 'display_order': 90, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:53.590171+05:30', 'updated_at': '2026-09-29T23:24:53.590190+05:30', 'agent_type': '22e700fe-df | POST 400 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/verify/ =&gt; {'registered_mobile_number': 'Registered Mobile (Bank) is required before approval.', 'is_pan_verified': 'PAN must be verified before approval.', 'is_bank_details_verified': 'Bank details must be verified before approval.'} | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agents/17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a/ =&gt; {'id': '17bcd4d6-2735-4ddb-b3d8-aaaeaf9cef4a', 'branch_code': 'CHE001', 'branch_name': 'Adyar, Chennai', 'agent_type_name': 'Private Limited Company', 'agent_channel_name': 'Internal Agent', 'referral_source_code': 'IN', 'referral_source_name': 'Internal (Sales Team)', 'referral_source_is_code_required': False, 'verified_by_user': None, 'category': 'Partner', 'documents': [{'document_code': 'pan_image', 'document_name': 'PAN Image', 'name': 'PAN Image', 'field': 'pan_image', 's3_key': '17bcd4d6- | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true =&gt; [{'id': '10bea8fd-2c9c-4703-9789-486491aa2e49', 'agent_type_name': 'Private Limited Company', 'field_code': 'cin_llpin', 'field_name': 'CIN / LLPIN Number', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': None, 'validation_message': None, 'placeholder': None, 'display_order': 90, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:53.590171+05:30', 'updated_at': '2026-09-29T23:24:53.590190+05:30', 'agent_type': '22e700fe-df | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/branches/?is_active=true =&gt; [{'id': '2e4b5706-6315-4f53-aa7c-f5aa545180fe', 'spoc_mailid': [{'name': 'panchakshari', 'mailid': 'panchu@gmail.com', 'department': 'finance'}, {'name': 'basavaraj', 'mailid': 'basav@gmail.com', 'department': 'branch user'}], 'zone': None, 'city_name': 'Bengaluru', 'state_name': 'karnataka', 'country_name': 'india', 'zone_name': None, 'zone_code': None, 'is_delete': False, 'created_at': '2026-01-31T17:04:05.342849+05:30', 'updated_at': '2026-10-09T18:20:11.863338+05:30', 'deleted_at': None, 'na | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-required-fields/?agent_type=22e700fe-df45-41b6-b72a-10a3506437f7&amp;is_active=true =&gt; [{'id': '10bea8fd-2c9c-4703-9789-486491aa2e49', 'agent_type_name': 'Private Limited Company', 'field_code': 'cin_llpin', 'field_name': 'CIN / LLPIN Number', 'section': 'profile', 'input_type': 'text', 'is_required': True, 'validation_regex': None, 'validation_message': None, 'placeholder': None, 'display_order': 90, 'options': None, 'is_active': True, 'is_delete': False, 'created_at': '2026-09-29T23:24:53.590171+05:30', 'updated_at': '2026-09-29T23:24:53.590190+05:30', 'agent_type': '22e700fe-df | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/referral-sources/ =&gt; [{'id': '0d59f0d0-acbc-428d-94df-65e894662f39', 'options': [], 'is_delete': False, 'created_at': '2026-03-09T14:29:29.839887+05:30', 'updated_at': '2026-03-09T14:29:29.839887+05:30', 'deleted_at': None, 'name': 'Corporate Referral', 'code': 'CR', 'description': 'Referral from corporate partners', 'is_active': True, 'is_code_required': False, 'requires_option': False, 'deleted_by': None, 'created_by': None, 'updated_by': None}, {'id': '3d3868af-83f1-4e1c-9c2d-6c367656b907', 'options': [], 'is_del | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/masters/agent-categories/ =&gt; [{'id': 'c221762a-5fe5-4c3e-b773-53aae4a7462d', 'is_delete': False, 'created_at': '2026-08-20T00:33:04.027484+05:30', 'updated_at': '2026-09-11T17:34:11.604215+05:30', 'deleted_at': None, 'category_name': 'Corporate', 'category_description': 'Corporate Partner', 'is_active': True, 'deleted_by': None, 'created_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93', 'updated_by': 'c3aa493a-4fb0-4c53-9d58-07cb691c0f93'}, {'id': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb', 'is_delete': False, 'created_at': '2026-07 | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-channels/ =&gt; [{'id': '0072498c-a181-481c-85ed-0ef2cf951a6e', 'code': 'EXTERNAL', 'name': 'External Agent', 'description': 'Agents who operate outside the organization (field / third-party agents)', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-17T09:53:25.309000+05:30', 'updated_at': '2026-01-24T13:05:19.593325+05:30'}, {'id': 'dee1f305-d140-4759-bb49-70fc94d8c848', 'code': 'INTERNAL', 'name': 'Internal Agent', 'description': 'Agents who operate within the organization (internal operations)', | GET 200 http://prithvifx-admin-backend-env-1.eba-aedqi5mv.ap-south-1.elasticbeanstalk.com/api/admin-agents/agent-types/ =&gt; [{'id': 'ec8d7645-535d-4a02-a2e6-059609a6cfe3', 'category_name': 'Partner', 'type_code': 'TPI', 'type_name': 'Individual', 'type_description': 'Individual agent operating as sole proprietor', 'is_active': True, 'is_delete': False, 'created_at': '2026-01-24T13:29:57.792000+05:30', 'updated_at': '2026-09-26T12:21:15.700380+05:30', 'category': 'c8a56c39-81c3-41c5-9f64-66cd20118dbb'}, {'id': 'ae4f60ef-acd3-4cc2-9d90-29a2cb3b1db2', 'category_name': 'Corporate', 'type_code': 'LLP', 'type_name': 'Limit | GET 200 htt</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>64.42</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>reports/screenshots/test_add_partner.png</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2026-10-13 18:39:21</t>
         </is>
       </c>
     </row>

</xml_diff>